<commit_message>
feat: user can export ICS as PDF
</commit_message>
<xml_diff>
--- a/procurement_documents/ICS Template.xlsx
+++ b/procurement_documents/ICS Template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BC06660-DFB7-44B0-B1E9-DD6DEAF69107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1E164C5-5DDA-41F0-AB90-D3EDDA3E44C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{28A639EE-9D7E-4335-A6BA-4B670CD55FAE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{28A639EE-9D7E-4335-A6BA-4B670CD55FAE}"/>
   </bookViews>
   <sheets>
     <sheet name="ICS" sheetId="1" r:id="rId1"/>
@@ -469,65 +469,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -545,12 +488,6 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -558,45 +495,15 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -606,12 +513,6 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -661,60 +562,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -725,17 +572,173 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1044,738 +1047,739 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31519EDA-B48E-45A4-93A1-DAFA93EE462A}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:N10723"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" customWidth="1"/>
-    <col min="2" max="2" width="5.85546875" customWidth="1"/>
-    <col min="3" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="10" style="85" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" customWidth="1"/>
+    <col min="3" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="30.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" style="34" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="6"/>
+      <c r="A1" s="81"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="86"/>
     </row>
     <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="87" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="10" t="s">
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="92"/>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="10" t="s">
+      <c r="B3" s="88"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="90" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="12"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="92"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="15"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="77"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="13" t="s">
+      <c r="B5" s="76"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="14"/>
-      <c r="H5" s="15"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="77"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="18"/>
+      <c r="B6" s="79"/>
+      <c r="C6" s="79"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="80"/>
+      <c r="F6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="80"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="25" t="s">
+      <c r="B7" s="57"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="26"/>
+      <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="31" t="s">
+      <c r="B8" s="60"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="91"/>
-      <c r="H8" s="92"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="62"/>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="34"/>
-      <c r="E9" s="35" t="s">
+      <c r="D9" s="66"/>
+      <c r="E9" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="36"/>
-      <c r="G9" s="37" t="s">
+      <c r="F9" s="68"/>
+      <c r="G9" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="38" t="s">
+      <c r="H9" s="73" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
-      <c r="B10" s="39"/>
-      <c r="C10" s="40" t="s">
+      <c r="A10" s="64"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="41"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="44"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="72"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="45"/>
-      <c r="B11" s="45"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="89"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="48"/>
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="54"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="93"/>
+      <c r="H11" s="11"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="45"/>
-      <c r="B12" s="45"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="89"/>
-      <c r="F12" s="90"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="49"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="45"/>
-      <c r="B13" s="45"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="89"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="50"/>
-      <c r="H13" s="49"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="45"/>
-      <c r="B14" s="45"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="89"/>
-      <c r="F14" s="90"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="49"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="13"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="45"/>
-      <c r="B15" s="45"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="89"/>
-      <c r="F15" s="90"/>
-      <c r="G15" s="47"/>
-      <c r="H15" s="49"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="13"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="51"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="89"/>
-      <c r="F16" s="90"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="49"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="51"/>
-      <c r="B17" s="45"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="89"/>
-      <c r="F17" s="90"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="49"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="13"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="45"/>
-      <c r="B18" s="53"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="89"/>
-      <c r="F18" s="90"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="49"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="13"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="54"/>
-      <c r="B19" s="53"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="89"/>
-      <c r="F19" s="90"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="49"/>
+      <c r="A19" s="21"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="54"/>
+      <c r="F19" s="55"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="13"/>
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="54"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="89"/>
-      <c r="F20" s="90"/>
-      <c r="G20" s="50"/>
-      <c r="H20" s="55"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="22"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="54"/>
-      <c r="B21" s="53"/>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="89"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="50"/>
-      <c r="H21" s="55"/>
+      <c r="A21" s="21"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="22"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="51"/>
-      <c r="B22" s="51"/>
-      <c r="C22" s="56"/>
-      <c r="D22" s="56"/>
-      <c r="E22" s="89"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="57"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="55"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="24"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="51"/>
-      <c r="B23" s="51"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="89"/>
-      <c r="F23" s="90"/>
-      <c r="G23" s="58"/>
-      <c r="H23" s="57"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="55"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="24"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="51"/>
-      <c r="B24" s="51"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="89"/>
-      <c r="F24" s="90"/>
-      <c r="G24" s="58"/>
-      <c r="H24" s="57"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="24"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="45"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="89"/>
-      <c r="F25" s="90"/>
-      <c r="G25" s="58"/>
-      <c r="H25" s="59"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="26"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="45"/>
-      <c r="B26" s="51"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="89"/>
-      <c r="F26" s="90"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="59"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="55"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="26"/>
     </row>
     <row r="27" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="45"/>
-      <c r="B27" s="53"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="89"/>
-      <c r="F27" s="90"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="59"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="54"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="26"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="45"/>
-      <c r="B28" s="53"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="89"/>
-      <c r="F28" s="90"/>
-      <c r="G28" s="58"/>
-      <c r="H28" s="59"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="54"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="26"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="53"/>
-      <c r="B29" s="45"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="89"/>
-      <c r="F29" s="90"/>
-      <c r="G29" s="58"/>
-      <c r="H29" s="59"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="54"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="26"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="53"/>
-      <c r="B30" s="45"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="89"/>
-      <c r="F30" s="90"/>
-      <c r="G30" s="58"/>
-      <c r="H30" s="61"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="54"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="28"/>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="53"/>
-      <c r="B31" s="45"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="89"/>
-      <c r="F31" s="90"/>
-      <c r="G31" s="58"/>
-      <c r="H31" s="61"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="54"/>
+      <c r="F31" s="55"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="28"/>
     </row>
     <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="53"/>
-      <c r="B32" s="45"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="89"/>
-      <c r="F32" s="90"/>
-      <c r="G32" s="58"/>
-      <c r="H32" s="61"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="54"/>
+      <c r="F32" s="55"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="28"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="45"/>
-      <c r="B33" s="45"/>
-      <c r="C33" s="46"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="89"/>
-      <c r="F33" s="90"/>
-      <c r="G33" s="58"/>
-      <c r="H33" s="61"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="54"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="28"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="45"/>
-      <c r="B34" s="45"/>
-      <c r="C34" s="46"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="89"/>
-      <c r="F34" s="90"/>
-      <c r="G34" s="58"/>
-      <c r="H34" s="59"/>
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="54"/>
+      <c r="F34" s="55"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="26"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="45"/>
-      <c r="B35" s="45"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="56"/>
-      <c r="E35" s="89"/>
-      <c r="F35" s="90"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="59"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="54"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="26"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="51"/>
-      <c r="B36" s="51"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="89"/>
-      <c r="F36" s="90"/>
-      <c r="G36" s="58"/>
-      <c r="H36" s="59"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="54"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="26"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="51"/>
-      <c r="B37" s="45"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="89"/>
-      <c r="F37" s="90"/>
-      <c r="G37" s="58"/>
-      <c r="H37" s="59"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="54"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="26"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="51"/>
-      <c r="B38" s="45"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="89"/>
-      <c r="F38" s="90"/>
-      <c r="G38" s="58"/>
-      <c r="H38" s="59"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="54"/>
+      <c r="F38" s="55"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="26"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="51"/>
-      <c r="B39" s="45"/>
-      <c r="C39" s="46"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="89"/>
-      <c r="F39" s="90"/>
-      <c r="G39" s="58"/>
-      <c r="H39" s="59"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="26"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="51"/>
-      <c r="B40" s="45"/>
-      <c r="C40" s="46"/>
-      <c r="D40" s="46"/>
-      <c r="E40" s="89"/>
-      <c r="F40" s="90"/>
-      <c r="G40" s="58"/>
-      <c r="H40" s="59"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="54"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="26"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="51"/>
-      <c r="B41" s="45"/>
-      <c r="C41" s="46"/>
-      <c r="D41" s="46"/>
-      <c r="E41" s="89"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="58"/>
-      <c r="H41" s="59"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="54"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="25"/>
+      <c r="H41" s="26"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="51"/>
-      <c r="B42" s="45"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="89"/>
-      <c r="F42" s="90"/>
-      <c r="G42" s="58"/>
-      <c r="H42" s="59"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="54"/>
+      <c r="F42" s="55"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="26"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="51"/>
-      <c r="B43" s="45"/>
-      <c r="C43" s="46"/>
-      <c r="D43" s="46"/>
-      <c r="E43" s="89"/>
-      <c r="F43" s="90"/>
-      <c r="G43" s="58"/>
-      <c r="H43" s="59"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="54"/>
+      <c r="F43" s="55"/>
+      <c r="G43" s="25"/>
+      <c r="H43" s="26"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="51"/>
-      <c r="B44" s="51"/>
-      <c r="C44" s="46"/>
-      <c r="D44" s="46"/>
-      <c r="E44" s="89"/>
-      <c r="F44" s="90"/>
-      <c r="G44" s="58"/>
-      <c r="H44" s="59"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="54"/>
+      <c r="F44" s="55"/>
+      <c r="G44" s="25"/>
+      <c r="H44" s="26"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="53"/>
-      <c r="B45" s="45"/>
-      <c r="C45" s="46"/>
-      <c r="D45" s="46"/>
-      <c r="E45" s="89"/>
-      <c r="F45" s="90"/>
-      <c r="G45" s="58"/>
-      <c r="H45" s="59"/>
+      <c r="A45" s="20"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="54"/>
+      <c r="F45" s="55"/>
+      <c r="G45" s="25"/>
+      <c r="H45" s="26"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="62"/>
-      <c r="B46" s="63"/>
-      <c r="C46" s="64"/>
-      <c r="D46" s="64"/>
-      <c r="E46" s="89"/>
-      <c r="F46" s="90"/>
-      <c r="G46" s="65"/>
-      <c r="H46" s="66"/>
+      <c r="A46" s="29"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="54"/>
+      <c r="F46" s="55"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="33"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="62"/>
-      <c r="B47" s="63"/>
-      <c r="C47" s="64"/>
-      <c r="D47" s="64"/>
-      <c r="E47" s="89"/>
-      <c r="F47" s="90"/>
-      <c r="G47" s="65"/>
-      <c r="H47" s="66"/>
+      <c r="A47" s="29"/>
+      <c r="B47" s="30"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="54"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="33"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="67"/>
-      <c r="F48" s="19" t="s">
+      <c r="B48" s="57"/>
+      <c r="C48" s="57"/>
+      <c r="D48" s="57"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="G48" s="20"/>
-      <c r="H48" s="68"/>
+      <c r="G48" s="57"/>
+      <c r="H48" s="58"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="69"/>
-      <c r="B49" s="70"/>
-      <c r="C49" s="70"/>
-      <c r="D49" s="70"/>
-      <c r="E49" s="70"/>
-      <c r="F49" s="69"/>
-      <c r="G49" s="70"/>
-      <c r="H49" s="71"/>
+      <c r="A49" s="38"/>
+      <c r="B49" s="39"/>
+      <c r="C49" s="39"/>
+      <c r="D49" s="39"/>
+      <c r="E49" s="39"/>
+      <c r="F49" s="38"/>
+      <c r="G49" s="39"/>
+      <c r="H49" s="46"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="72"/>
-      <c r="B50" s="73"/>
-      <c r="C50" s="73"/>
-      <c r="D50" s="73"/>
-      <c r="E50" s="73"/>
-      <c r="F50" s="72"/>
-      <c r="G50" s="73"/>
-      <c r="H50" s="74"/>
+      <c r="A50" s="49"/>
+      <c r="B50" s="50"/>
+      <c r="C50" s="50"/>
+      <c r="D50" s="50"/>
+      <c r="E50" s="50"/>
+      <c r="F50" s="49"/>
+      <c r="G50" s="50"/>
+      <c r="H50" s="51"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A51" s="69"/>
-      <c r="B51" s="70"/>
-      <c r="C51" s="70"/>
-      <c r="D51" s="70"/>
-      <c r="E51" s="70"/>
-      <c r="F51" s="69" t="s">
+      <c r="A51" s="38"/>
+      <c r="B51" s="39"/>
+      <c r="C51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="G51" s="70"/>
-      <c r="H51" s="71"/>
+      <c r="G51" s="39"/>
+      <c r="H51" s="46"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="B52" s="76"/>
-      <c r="C52" s="76"/>
-      <c r="D52" s="76"/>
-      <c r="E52" s="76"/>
-      <c r="F52" s="72"/>
-      <c r="G52" s="73"/>
-      <c r="H52" s="74"/>
+      <c r="B52" s="48"/>
+      <c r="C52" s="48"/>
+      <c r="D52" s="48"/>
+      <c r="E52" s="48"/>
+      <c r="F52" s="49"/>
+      <c r="G52" s="50"/>
+      <c r="H52" s="51"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A53" s="77"/>
-      <c r="B53" s="78"/>
-      <c r="C53" s="78"/>
-      <c r="D53" s="78"/>
-      <c r="E53" s="78"/>
-      <c r="F53" s="69" t="s">
+      <c r="A53" s="52"/>
+      <c r="B53" s="53"/>
+      <c r="C53" s="53"/>
+      <c r="D53" s="53"/>
+      <c r="E53" s="53"/>
+      <c r="F53" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="G53" s="70"/>
-      <c r="H53" s="71"/>
+      <c r="G53" s="39"/>
+      <c r="H53" s="46"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="69" t="s">
+      <c r="A54" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="B54" s="70"/>
-      <c r="C54" s="70"/>
-      <c r="D54" s="70"/>
-      <c r="E54" s="70"/>
-      <c r="F54" s="79"/>
-      <c r="G54" s="80"/>
-      <c r="H54" s="81"/>
+      <c r="B54" s="39"/>
+      <c r="C54" s="39"/>
+      <c r="D54" s="39"/>
+      <c r="E54" s="39"/>
+      <c r="F54" s="40"/>
+      <c r="G54" s="41"/>
+      <c r="H54" s="42"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A55" s="82"/>
-      <c r="B55" s="83"/>
-      <c r="C55" s="83"/>
-      <c r="D55" s="83"/>
-      <c r="E55" s="83"/>
-      <c r="F55" s="82" t="s">
+      <c r="A55" s="43"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="44"/>
+      <c r="F55" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="G55" s="83"/>
-      <c r="H55" s="84"/>
+      <c r="G55" s="44"/>
+      <c r="H55" s="45"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N61" s="86"/>
+      <c r="N61" s="35"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N62" s="86"/>
+      <c r="N62" s="35"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N63" s="86"/>
+      <c r="N63" s="35"/>
     </row>
     <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N64" s="86"/>
+      <c r="N64" s="35"/>
     </row>
     <row r="65" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N65" s="86"/>
+      <c r="N65" s="35"/>
     </row>
     <row r="66" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N66" s="86"/>
+      <c r="N66" s="35"/>
     </row>
     <row r="67" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N67" s="86"/>
+      <c r="N67" s="35"/>
     </row>
     <row r="68" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N68" s="86"/>
+      <c r="N68" s="35"/>
     </row>
     <row r="69" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N69" s="86"/>
+      <c r="N69" s="35"/>
     </row>
     <row r="70" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N70" s="87"/>
+      <c r="N70" s="36"/>
     </row>
     <row r="71" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N71" s="86"/>
+      <c r="N71" s="35"/>
     </row>
     <row r="72" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N72" s="86"/>
+      <c r="N72" s="35"/>
     </row>
     <row r="73" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N73" s="86"/>
+      <c r="N73" s="35"/>
     </row>
     <row r="74" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N74" s="86"/>
+      <c r="N74" s="35"/>
     </row>
     <row r="75" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N75" s="86"/>
+      <c r="N75" s="35"/>
     </row>
     <row r="76" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N76" s="86"/>
+      <c r="N76" s="35"/>
     </row>
     <row r="77" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N77" s="86"/>
+      <c r="N77" s="35"/>
     </row>
     <row r="78" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N78" s="86"/>
+      <c r="N78" s="35"/>
     </row>
     <row r="79" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N79" s="86"/>
+      <c r="N79" s="35"/>
     </row>
     <row r="80" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N80" s="86"/>
+      <c r="N80" s="35"/>
     </row>
     <row r="81" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N81" s="86"/>
+      <c r="N81" s="35"/>
     </row>
     <row r="82" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N82" s="86"/>
+      <c r="N82" s="35"/>
     </row>
     <row r="83" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N83" s="86"/>
+      <c r="N83" s="35"/>
     </row>
     <row r="84" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N84" s="86"/>
+      <c r="N84" s="35"/>
     </row>
     <row r="85" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N85" s="86"/>
+      <c r="N85" s="35"/>
     </row>
     <row r="86" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N86" s="86"/>
+      <c r="N86" s="35"/>
     </row>
     <row r="87" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N87" s="86"/>
+      <c r="N87" s="35"/>
     </row>
     <row r="88" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N88" s="86"/>
+      <c r="N88" s="35"/>
     </row>
     <row r="89" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N89" s="86"/>
+      <c r="N89" s="35"/>
     </row>
     <row r="90" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N90" s="86"/>
+      <c r="N90" s="35"/>
     </row>
     <row r="91" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N91" s="86"/>
+      <c r="N91" s="35"/>
     </row>
     <row r="92" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N92" s="86"/>
+      <c r="N92" s="35"/>
     </row>
     <row r="93" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N93" s="86"/>
+      <c r="N93" s="35"/>
     </row>
     <row r="94" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N94" s="86"/>
+      <c r="N94" s="35"/>
     </row>
     <row r="95" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N95" s="86"/>
+      <c r="N95" s="35"/>
     </row>
     <row r="96" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N96" s="86"/>
+      <c r="N96" s="35"/>
     </row>
     <row r="97" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N97" s="86"/>
+      <c r="N97" s="35"/>
     </row>
     <row r="98" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N98" s="86"/>
+      <c r="N98" s="35"/>
     </row>
     <row r="100" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N100" s="88"/>
+      <c r="N100" s="37"/>
     </row>
     <row r="119" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="174" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1985,30 +1989,35 @@
     <row r="10723" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="E9:F10"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="F49:H49"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="F51:H51"/>
     <mergeCell ref="A55:E55"/>
     <mergeCell ref="F55:H55"/>
     <mergeCell ref="E11:F11"/>
@@ -2025,40 +2034,35 @@
     <mergeCell ref="F53:H53"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="F54:H54"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="E30:F30"/>
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="E22:F22"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:F10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E47:F47"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39300000000000002" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2067,772 +2071,773 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F81A5BCB-5285-45BC-AA2A-0BC2370CAAE6}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:N10723"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" customWidth="1"/>
-    <col min="2" max="2" width="5.85546875" customWidth="1"/>
-    <col min="3" max="4" width="10.85546875" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="10" style="85" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" customWidth="1"/>
+    <col min="3" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="30.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" style="34" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="6"/>
+      <c r="A1" s="81"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="83"/>
+      <c r="F1" s="84"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="86"/>
     </row>
     <row r="2" spans="1:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="87" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="10" t="s">
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="92"/>
     </row>
     <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="10" t="s">
+      <c r="B3" s="88"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="90" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="12"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="92"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="75" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="15"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="75"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="77"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="75" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="13" t="s">
+      <c r="B5" s="76"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="14"/>
-      <c r="H5" s="15"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="77"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="18"/>
+      <c r="B6" s="79"/>
+      <c r="C6" s="79"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="80"/>
+      <c r="F6" s="78"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="80"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="20"/>
-      <c r="C7" s="21" t="s">
+      <c r="B7" s="57"/>
+      <c r="C7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="25" t="s">
+      <c r="D7" s="3"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="26" t="s">
+      <c r="H7" s="7" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+      <c r="A8" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="28"/>
-      <c r="C8" s="29" t="s">
+      <c r="B8" s="60"/>
+      <c r="C8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="30"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="31" t="s">
+      <c r="D8" s="9"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="91" t="s">
+      <c r="G8" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="92"/>
+      <c r="H8" s="62"/>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="34"/>
-      <c r="E9" s="35" t="s">
+      <c r="D9" s="66"/>
+      <c r="E9" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="36"/>
-      <c r="G9" s="37" t="s">
+      <c r="F9" s="68"/>
+      <c r="G9" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="38" t="s">
+      <c r="H9" s="73" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
-      <c r="B10" s="39"/>
-      <c r="C10" s="40" t="s">
+      <c r="A10" s="64"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="41"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="44"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="70"/>
+      <c r="G10" s="72"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="45" t="s">
+      <c r="A11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="45" t="s">
+      <c r="B11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="89" t="s">
+      <c r="E11" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="F11" s="90"/>
-      <c r="G11" s="47" t="s">
+      <c r="F11" s="55"/>
+      <c r="G11" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="H11" s="48" t="s">
+      <c r="H11" s="11" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="45"/>
-      <c r="B12" s="45"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="89"/>
-      <c r="F12" s="90"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="49"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="45"/>
-      <c r="B13" s="45"/>
-      <c r="C13" s="46"/>
-      <c r="D13" s="46"/>
-      <c r="E13" s="89"/>
-      <c r="F13" s="90"/>
-      <c r="G13" s="50"/>
-      <c r="H13" s="49"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="45"/>
-      <c r="B14" s="45"/>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="89"/>
-      <c r="F14" s="90"/>
-      <c r="G14" s="47"/>
-      <c r="H14" s="49"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="13"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="45"/>
-      <c r="B15" s="45"/>
-      <c r="C15" s="46"/>
-      <c r="D15" s="46"/>
-      <c r="E15" s="89"/>
-      <c r="F15" s="90"/>
-      <c r="G15" s="47"/>
-      <c r="H15" s="49"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="13"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="51"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="89"/>
-      <c r="F16" s="90"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="49"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="51"/>
-      <c r="B17" s="45"/>
-      <c r="C17" s="46"/>
-      <c r="D17" s="46"/>
-      <c r="E17" s="89"/>
-      <c r="F17" s="90"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="49"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="13"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="45"/>
-      <c r="B18" s="53"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="89"/>
-      <c r="F18" s="90"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="49"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="13"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="54"/>
-      <c r="B19" s="53"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="89"/>
-      <c r="F19" s="90"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="49"/>
+      <c r="A19" s="21"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="54"/>
+      <c r="F19" s="55"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="13"/>
     </row>
     <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="54"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="89"/>
-      <c r="F20" s="90"/>
-      <c r="G20" s="50"/>
-      <c r="H20" s="55"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="55"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="22"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="54"/>
-      <c r="B21" s="53"/>
-      <c r="C21" s="56"/>
-      <c r="D21" s="56"/>
-      <c r="E21" s="89"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="50"/>
-      <c r="H21" s="55"/>
+      <c r="A21" s="21"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="22"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="51"/>
-      <c r="B22" s="51"/>
-      <c r="C22" s="56"/>
-      <c r="D22" s="56"/>
-      <c r="E22" s="89"/>
-      <c r="F22" s="90"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="57"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="55"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="24"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="51"/>
-      <c r="B23" s="51"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="56"/>
-      <c r="E23" s="89"/>
-      <c r="F23" s="90"/>
-      <c r="G23" s="58"/>
-      <c r="H23" s="57"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="55"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="24"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="51"/>
-      <c r="B24" s="51"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="56"/>
-      <c r="E24" s="89"/>
-      <c r="F24" s="90"/>
-      <c r="G24" s="58"/>
-      <c r="H24" s="57"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="24"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="45"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="89"/>
-      <c r="F25" s="90"/>
-      <c r="G25" s="58"/>
-      <c r="H25" s="59"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="26"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="45"/>
-      <c r="B26" s="51"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="89"/>
-      <c r="F26" s="90"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="59"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="54"/>
+      <c r="F26" s="55"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="26"/>
     </row>
     <row r="27" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="45"/>
-      <c r="B27" s="53"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="89"/>
-      <c r="F27" s="90"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="59"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="54"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="26"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="45"/>
-      <c r="B28" s="53"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="89"/>
-      <c r="F28" s="90"/>
-      <c r="G28" s="58"/>
-      <c r="H28" s="59"/>
+      <c r="A28" s="14"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="54"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="26"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="53"/>
-      <c r="B29" s="45"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="56"/>
-      <c r="E29" s="89"/>
-      <c r="F29" s="90"/>
-      <c r="G29" s="58"/>
-      <c r="H29" s="59"/>
+      <c r="A29" s="20"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="54"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="26"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="53"/>
-      <c r="B30" s="45"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="89"/>
-      <c r="F30" s="90"/>
-      <c r="G30" s="58"/>
-      <c r="H30" s="61"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="54"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="28"/>
     </row>
     <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="53"/>
-      <c r="B31" s="45"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="89"/>
-      <c r="F31" s="90"/>
-      <c r="G31" s="58"/>
-      <c r="H31" s="61"/>
+      <c r="A31" s="20"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="54"/>
+      <c r="F31" s="55"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="28"/>
     </row>
     <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="53"/>
-      <c r="B32" s="45"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="89"/>
-      <c r="F32" s="90"/>
-      <c r="G32" s="58"/>
-      <c r="H32" s="61"/>
+      <c r="A32" s="20"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="54"/>
+      <c r="F32" s="55"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="28"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="45"/>
-      <c r="B33" s="45"/>
-      <c r="C33" s="46"/>
-      <c r="D33" s="56"/>
-      <c r="E33" s="89"/>
-      <c r="F33" s="90"/>
-      <c r="G33" s="58"/>
-      <c r="H33" s="61"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="54"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="28"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="45"/>
-      <c r="B34" s="45"/>
-      <c r="C34" s="46"/>
-      <c r="D34" s="46"/>
-      <c r="E34" s="89"/>
-      <c r="F34" s="90"/>
-      <c r="G34" s="58"/>
-      <c r="H34" s="59"/>
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="54"/>
+      <c r="F34" s="55"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="26"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="45"/>
-      <c r="B35" s="45"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="56"/>
-      <c r="E35" s="89"/>
-      <c r="F35" s="90"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="59"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="54"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="26"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="51"/>
-      <c r="B36" s="51"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="46"/>
-      <c r="E36" s="89"/>
-      <c r="F36" s="90"/>
-      <c r="G36" s="58"/>
-      <c r="H36" s="59"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="54"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="26"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="51"/>
-      <c r="B37" s="45"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="89"/>
-      <c r="F37" s="90"/>
-      <c r="G37" s="58"/>
-      <c r="H37" s="59"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="54"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="25"/>
+      <c r="H37" s="26"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="51"/>
-      <c r="B38" s="45"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="46"/>
-      <c r="E38" s="89"/>
-      <c r="F38" s="90"/>
-      <c r="G38" s="58"/>
-      <c r="H38" s="59"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="54"/>
+      <c r="F38" s="55"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="26"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="51"/>
-      <c r="B39" s="45"/>
-      <c r="C39" s="46"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="89"/>
-      <c r="F39" s="90"/>
-      <c r="G39" s="58"/>
-      <c r="H39" s="59"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="55"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="26"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="51"/>
-      <c r="B40" s="45"/>
-      <c r="C40" s="46"/>
-      <c r="D40" s="46"/>
-      <c r="E40" s="89"/>
-      <c r="F40" s="90"/>
-      <c r="G40" s="58"/>
-      <c r="H40" s="59"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="54"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="25"/>
+      <c r="H40" s="26"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="51"/>
-      <c r="B41" s="45"/>
-      <c r="C41" s="46"/>
-      <c r="D41" s="46"/>
-      <c r="E41" s="89"/>
-      <c r="F41" s="90"/>
-      <c r="G41" s="58"/>
-      <c r="H41" s="59"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="54"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="25"/>
+      <c r="H41" s="26"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="51"/>
-      <c r="B42" s="45"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="89"/>
-      <c r="F42" s="90"/>
-      <c r="G42" s="58"/>
-      <c r="H42" s="59"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="54"/>
+      <c r="F42" s="55"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="26"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="51"/>
-      <c r="B43" s="45"/>
-      <c r="C43" s="46"/>
-      <c r="D43" s="46"/>
-      <c r="E43" s="89"/>
-      <c r="F43" s="90"/>
-      <c r="G43" s="58"/>
-      <c r="H43" s="59"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="54"/>
+      <c r="F43" s="55"/>
+      <c r="G43" s="25"/>
+      <c r="H43" s="26"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="51"/>
-      <c r="B44" s="51"/>
-      <c r="C44" s="46"/>
-      <c r="D44" s="46"/>
-      <c r="E44" s="89"/>
-      <c r="F44" s="90"/>
-      <c r="G44" s="58"/>
-      <c r="H44" s="59"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="54"/>
+      <c r="F44" s="55"/>
+      <c r="G44" s="25"/>
+      <c r="H44" s="26"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="53"/>
-      <c r="B45" s="45"/>
-      <c r="C45" s="46"/>
-      <c r="D45" s="46"/>
-      <c r="E45" s="89"/>
-      <c r="F45" s="90"/>
-      <c r="G45" s="58"/>
-      <c r="H45" s="59"/>
+      <c r="A45" s="20"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="54"/>
+      <c r="F45" s="55"/>
+      <c r="G45" s="25"/>
+      <c r="H45" s="26"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="62"/>
-      <c r="B46" s="63"/>
-      <c r="C46" s="64"/>
-      <c r="D46" s="64"/>
-      <c r="E46" s="89"/>
-      <c r="F46" s="90"/>
-      <c r="G46" s="65"/>
-      <c r="H46" s="66"/>
+      <c r="A46" s="29"/>
+      <c r="B46" s="30"/>
+      <c r="C46" s="31"/>
+      <c r="D46" s="31"/>
+      <c r="E46" s="54"/>
+      <c r="F46" s="55"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="33"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="62"/>
-      <c r="B47" s="63"/>
-      <c r="C47" s="64"/>
-      <c r="D47" s="64"/>
-      <c r="E47" s="89"/>
-      <c r="F47" s="90"/>
-      <c r="G47" s="65"/>
-      <c r="H47" s="66"/>
+      <c r="A47" s="29"/>
+      <c r="B47" s="30"/>
+      <c r="C47" s="31"/>
+      <c r="D47" s="31"/>
+      <c r="E47" s="54"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="33"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
+      <c r="A48" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="67"/>
-      <c r="F48" s="19" t="s">
+      <c r="B48" s="57"/>
+      <c r="C48" s="57"/>
+      <c r="D48" s="57"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="G48" s="20"/>
-      <c r="H48" s="68"/>
+      <c r="G48" s="57"/>
+      <c r="H48" s="58"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="69"/>
-      <c r="B49" s="70"/>
-      <c r="C49" s="70"/>
-      <c r="D49" s="70"/>
-      <c r="E49" s="70"/>
-      <c r="F49" s="69"/>
-      <c r="G49" s="70"/>
-      <c r="H49" s="71"/>
+      <c r="A49" s="38"/>
+      <c r="B49" s="39"/>
+      <c r="C49" s="39"/>
+      <c r="D49" s="39"/>
+      <c r="E49" s="39"/>
+      <c r="F49" s="38"/>
+      <c r="G49" s="39"/>
+      <c r="H49" s="46"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="72" t="s">
+      <c r="A50" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="B50" s="73"/>
-      <c r="C50" s="73"/>
-      <c r="D50" s="73"/>
-      <c r="E50" s="73"/>
-      <c r="F50" s="72" t="s">
+      <c r="B50" s="50"/>
+      <c r="C50" s="50"/>
+      <c r="D50" s="50"/>
+      <c r="E50" s="50"/>
+      <c r="F50" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="G50" s="73"/>
-      <c r="H50" s="74"/>
+      <c r="G50" s="50"/>
+      <c r="H50" s="51"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A51" s="69" t="s">
+      <c r="A51" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="B51" s="70"/>
-      <c r="C51" s="70"/>
-      <c r="D51" s="70"/>
-      <c r="E51" s="70"/>
-      <c r="F51" s="69" t="s">
+      <c r="B51" s="39"/>
+      <c r="C51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="G51" s="70"/>
-      <c r="H51" s="71"/>
+      <c r="G51" s="39"/>
+      <c r="H51" s="46"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="B52" s="76"/>
-      <c r="C52" s="76"/>
-      <c r="D52" s="76"/>
-      <c r="E52" s="76"/>
-      <c r="F52" s="72" t="s">
+      <c r="B52" s="48"/>
+      <c r="C52" s="48"/>
+      <c r="D52" s="48"/>
+      <c r="E52" s="48"/>
+      <c r="F52" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="G52" s="73"/>
-      <c r="H52" s="74"/>
+      <c r="G52" s="50"/>
+      <c r="H52" s="51"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A53" s="77" t="s">
+      <c r="A53" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="B53" s="78"/>
-      <c r="C53" s="78"/>
-      <c r="D53" s="78"/>
-      <c r="E53" s="78"/>
-      <c r="F53" s="69" t="s">
+      <c r="B53" s="53"/>
+      <c r="C53" s="53"/>
+      <c r="D53" s="53"/>
+      <c r="E53" s="53"/>
+      <c r="F53" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="G53" s="70"/>
-      <c r="H53" s="71"/>
+      <c r="G53" s="39"/>
+      <c r="H53" s="46"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A54" s="69" t="s">
+      <c r="A54" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="B54" s="70"/>
-      <c r="C54" s="70"/>
-      <c r="D54" s="70"/>
-      <c r="E54" s="70"/>
-      <c r="F54" s="79" t="s">
+      <c r="B54" s="39"/>
+      <c r="C54" s="39"/>
+      <c r="D54" s="39"/>
+      <c r="E54" s="39"/>
+      <c r="F54" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="G54" s="80"/>
-      <c r="H54" s="81"/>
+      <c r="G54" s="41"/>
+      <c r="H54" s="42"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A55" s="82"/>
-      <c r="B55" s="83"/>
-      <c r="C55" s="83"/>
-      <c r="D55" s="83"/>
-      <c r="E55" s="83"/>
-      <c r="F55" s="82" t="s">
+      <c r="A55" s="43"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="E55" s="44"/>
+      <c r="F55" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="G55" s="83"/>
-      <c r="H55" s="84"/>
+      <c r="G55" s="44"/>
+      <c r="H55" s="45"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N61" s="86"/>
+      <c r="N61" s="35"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N62" s="86"/>
+      <c r="N62" s="35"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N63" s="86"/>
+      <c r="N63" s="35"/>
     </row>
     <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N64" s="86"/>
+      <c r="N64" s="35"/>
     </row>
     <row r="65" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N65" s="86"/>
+      <c r="N65" s="35"/>
     </row>
     <row r="66" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N66" s="86"/>
+      <c r="N66" s="35"/>
     </row>
     <row r="67" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N67" s="86"/>
+      <c r="N67" s="35"/>
     </row>
     <row r="68" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N68" s="86"/>
+      <c r="N68" s="35"/>
     </row>
     <row r="69" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N69" s="86"/>
+      <c r="N69" s="35"/>
     </row>
     <row r="70" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N70" s="87"/>
+      <c r="N70" s="36"/>
     </row>
     <row r="71" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N71" s="86"/>
+      <c r="N71" s="35"/>
     </row>
     <row r="72" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N72" s="86"/>
+      <c r="N72" s="35"/>
     </row>
     <row r="73" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N73" s="86"/>
+      <c r="N73" s="35"/>
     </row>
     <row r="74" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N74" s="86"/>
+      <c r="N74" s="35"/>
     </row>
     <row r="75" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N75" s="86"/>
+      <c r="N75" s="35"/>
     </row>
     <row r="76" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N76" s="86"/>
+      <c r="N76" s="35"/>
     </row>
     <row r="77" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N77" s="86"/>
+      <c r="N77" s="35"/>
     </row>
     <row r="78" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N78" s="86"/>
+      <c r="N78" s="35"/>
     </row>
     <row r="79" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N79" s="86"/>
+      <c r="N79" s="35"/>
     </row>
     <row r="80" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N80" s="86"/>
+      <c r="N80" s="35"/>
     </row>
     <row r="81" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N81" s="86"/>
+      <c r="N81" s="35"/>
     </row>
     <row r="82" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N82" s="86"/>
+      <c r="N82" s="35"/>
     </row>
     <row r="83" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N83" s="86"/>
+      <c r="N83" s="35"/>
     </row>
     <row r="84" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N84" s="86"/>
+      <c r="N84" s="35"/>
     </row>
     <row r="85" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N85" s="86"/>
+      <c r="N85" s="35"/>
     </row>
     <row r="86" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N86" s="86"/>
+      <c r="N86" s="35"/>
     </row>
     <row r="87" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N87" s="86"/>
+      <c r="N87" s="35"/>
     </row>
     <row r="88" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N88" s="86"/>
+      <c r="N88" s="35"/>
     </row>
     <row r="89" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N89" s="86"/>
+      <c r="N89" s="35"/>
     </row>
     <row r="90" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N90" s="86"/>
+      <c r="N90" s="35"/>
     </row>
     <row r="91" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N91" s="86"/>
+      <c r="N91" s="35"/>
     </row>
     <row r="92" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N92" s="86"/>
+      <c r="N92" s="35"/>
     </row>
     <row r="93" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N93" s="86"/>
+      <c r="N93" s="35"/>
     </row>
     <row r="94" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N94" s="86"/>
+      <c r="N94" s="35"/>
     </row>
     <row r="95" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N95" s="86"/>
+      <c r="N95" s="35"/>
     </row>
     <row r="96" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N96" s="86"/>
+      <c r="N96" s="35"/>
     </row>
     <row r="97" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N97" s="86"/>
+      <c r="N97" s="35"/>
     </row>
     <row r="98" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N98" s="86"/>
+      <c r="N98" s="35"/>
     </row>
     <row r="100" spans="14:14" x14ac:dyDescent="0.25">
-      <c r="N100" s="88"/>
+      <c r="N100" s="37"/>
     </row>
     <row r="119" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="174" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3042,6 +3047,70 @@
     <row r="10723" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="F48:H48"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="F49:H49"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="F54:H54"/>
     <mergeCell ref="A55:E55"/>
@@ -3052,70 +3121,6 @@
     <mergeCell ref="F52:H52"/>
     <mergeCell ref="A53:E53"/>
     <mergeCell ref="F53:H53"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="A48:D48"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.39300000000000002" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>